<commit_message>
Complete business rollout boundaries
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R4202833440fe474e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R4ff0f0806c154745"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -407,25 +407,33 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>完成条件</x:v>
+        <x:v>实施回退</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>两个Chart可由Helm处理，四种状态清单与合同闭合，三张业务决策表和证据范围表可按输入复算</x:v>
+        <x:v>实际变更窗口前重采集所有权与存储状态；条件回退时保留旧版本served并继续bridge，观察转换失败数和对象重写进度，恢复后另排窗口</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="5" t="str">
+        <x:v>完成条件</x:v>
+      </x:c>
+      <x:c r="B18" s="5" t="str">
+        <x:v>两个Chart可由Helm处理，四种状态清单与合同闭合，三张业务决策表和证据范围表可按输入复算</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="5" t="str">
         <x:v>可验证点</x:v>
       </x:c>
-      <x:c r="B18" s="5" t="str">
+      <x:c r="B19" s="5" t="str">
         <x:v>Chart名称、对象集合、API版本、served与storage布尔值、keep、conversion引用、状态枚举、阶段顺序和窗口主键</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="15" hidden="0" customHeight="1">
-      <x:c r="A19" s="6" t="str">
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="6" t="str">
         <x:v>不适合作为评分点的内容</x:v>
       </x:c>
-      <x:c r="B19" s="6" t="str">
+      <x:c r="B20" s="6" t="str">
         <x:v>YAML键序、文档顺序、模板拆分、注释、CSV行序、临时路径和文字排版</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Publish final Q2394 Helm reproduction
</commit_message>
<xml_diff>
--- a/task/任务规格转化.xlsx
+++ b/task/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="R4ff0f0806c154745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格" sheetId="1" r:id="Rd47a5a8bae724034"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -346,7 +346,7 @@
         <x:v>核心操作链</x:v>
       </x:c>
       <x:c r="B9" s="5" t="str">
-        <x:v>读取合同与快照→拆开Chart边界→渲染四种状态→检查对象与引用→判断所有权→判断退场→编排窗口</x:v>
+        <x:v>读取合同与发布记录→拆开Chart边界→渲染四种配置→检查对象与引用→判断所有权→安排版本切换→编排维护窗</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
@@ -383,10 +383,10 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="5" t="str">
-        <x:v>退场条件</x:v>
+        <x:v>切换条件</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>所有权READY、对象全部重写、转换失败为0且storedVersions精确等于v1时允许prune与steady</x:v>
+        <x:v>所有权READY、对象全部重写、转换失败为0且storedVersions精确等于v1时安排prune与steady</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -399,18 +399,18 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="5" t="str">
-        <x:v>证据口径</x:v>
+        <x:v>材料时点</x:v>
       </x:c>
       <x:c r="B16" s="5" t="str">
-        <x:v>输入CSV是离线快照，Helm输出是静态候选清单，均不代表集群实时运行状态</x:v>
+        <x:v>输入CSV记录交接材料的采集时间，值班发布人在维护窗前复查所有权与存储状态</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="5" t="str">
-        <x:v>实施回退</x:v>
+        <x:v>窗口处理</x:v>
       </x:c>
       <x:c r="B17" s="5" t="str">
-        <x:v>实际变更窗口前重采集所有权与存储状态；条件回退时保留旧版本served并继续bridge，观察转换失败数和对象重写进度，恢复后另排窗口</x:v>
+        <x:v>手续未齐或存储状态变化的集群保留additive和bridge，其他集群按合同顺序进入后续阶段</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">

</xml_diff>